<commit_message>
feat: rename the company and regenerate the corpus
Widget Makers Incorporated shares its name with a real manufacturer, and
several names invented inside the corpus did too. The generation prompts,
roster, and office guidance now name Main St Widget Foundry LLC, keep its
products deliberately vague, and forbid real company and product names.

The transcripts, office files, and store are regenerated, with every
invented name checked against a web search and replaced where it was
real. The tests, README examples, frontend fixtures, and the record of
planted imperfections follow the new corpus.

Closes #122
</commit_message>
<xml_diff>
--- a/data/office/support-ticket-sla-log.xlsx
+++ b/data/office/support-ticket-sla-log.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resolved Tickets" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resolved Tickets" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Tickets" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -427,19 +429,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="47" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
   </cols>
@@ -514,32 +516,32 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Fenwick Aggregates</t>
+          <t>Ivelmoor Group</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Unit fails self-test on power-up</t>
+          <t>RS-485 termination setting unclear</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>46023</v>
+        <v>46024</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>46027</v>
+        <v>46026</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>5</v>
@@ -551,12 +553,12 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -568,32 +570,32 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Harrowgate Cement</t>
+          <t>Quennick</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Intermittent signal dropout</t>
+          <t>Clock drift between units</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>46027</v>
+        <v>46025</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>46037</v>
+        <v>46031</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>10</v>
@@ -605,12 +607,12 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Sofia</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -622,35 +624,35 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Fenwick Aggregates</t>
+          <t>Trellisar</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Output chatter near target edge</t>
+          <t>Request for operating environment spec</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
+        <v>46027</v>
+      </c>
+      <c r="G4" s="3" t="n">
         <v>46029</v>
       </c>
-      <c r="G4" s="3" t="n">
-        <v>46033</v>
-      </c>
       <c r="H4" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -664,7 +666,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -676,35 +678,35 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Fenwick Aggregates</t>
+          <t>Tharnwick Rail</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Replacement mounting bracket request</t>
+          <t>Firmware update fails at 80 percent</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>46031</v>
+        <v>46029</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>46034</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
@@ -713,12 +715,12 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -730,17 +732,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Kessler Paper Mill</t>
+          <t>Tessivex</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Reading drift after ambient temperature rise</t>
+          <t>Slow response on serial polling</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -749,16 +751,16 @@
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>46031</v>
+        <v>46032</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>46035</v>
+        <v>46038</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -767,12 +769,12 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -784,35 +786,35 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Thornbury Power</t>
+          <t>Pemberlith Foods</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Echo loss on foam surface</t>
+          <t>Unit fails self-test after power interruption</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>46031</v>
+        <v>46035</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>46033</v>
+        <v>46044</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
@@ -838,35 +840,35 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Barrow Tide Ports</t>
+          <t>Quennick</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Configuration tool connection error</t>
+          <t>Request for replacement terminal plugs</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
         <v>46034</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>46035</v>
+        <v>46037</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -875,12 +877,12 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -892,49 +894,49 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Grayson Textiles</t>
+          <t>Pemberlith Foods</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Reading drift after ambient temperature rise</t>
+          <t>Question on mounting orientation</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>46043</v>
+        <v>46036</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>46047</v>
+        <v>46048</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Marcus</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -946,35 +948,35 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Sable Creek Gas</t>
+          <t>Pemberlith Foods</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Calibration offset after install</t>
+          <t>Unit fails self-test after power interruption</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46045</v>
+        <v>46038</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>46049</v>
+        <v>46039</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
@@ -988,7 +990,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1000,35 +1002,35 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Thornbury Power</t>
+          <t>Pemberlith Foods</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Intermittent signal dropout</t>
+          <t>Configuration lost after firmware update</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="F11" s="3" t="n">
-        <v>46049</v>
+        <v>46041</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>46053</v>
+        <v>46043</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
@@ -1037,12 +1039,12 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1054,29 +1056,29 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Grayson Textiles</t>
+          <t>Sorrelby Water</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Firmware update failed mid-flash</t>
+          <t>Unit reboots under brownout</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F12" s="3" t="n">
-        <v>46055</v>
+        <v>46042</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>46059</v>
+        <v>46046</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>4</v>
@@ -1091,12 +1093,12 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1108,49 +1110,49 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Stanmore Polymers</t>
+          <t>Tharnwick Rail</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Echo loss on foam surface</t>
+          <t>Bus address conflict on commissioning</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F13" s="3" t="n">
-        <v>46059</v>
+        <v>46044</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>46063</v>
+        <v>46053</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Sofia</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1162,35 +1164,35 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Delvecchio Packaging</t>
+          <t>Callowmere Packaging</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Output chatter near target edge</t>
+          <t>Unit reboots under brownout</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F14" s="3" t="n">
-        <v>46063</v>
+        <v>46047</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>46069</v>
+        <v>46049</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
@@ -1199,12 +1201,12 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1216,49 +1218,49 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Sable Creek Gas</t>
+          <t>Ivelmoor Group</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>4-20 mA output offset</t>
+          <t>Firmware update fails at 80 percent</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F15" s="3" t="n">
-        <v>46065</v>
+        <v>46049</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>46069</v>
+        <v>46058</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Sofia</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1270,49 +1272,49 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Sable Creek Gas</t>
+          <t>Kilnwarden Utilities</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Firmware update failed mid-flash</t>
+          <t>Firmware version query over API</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
-        <v>46066</v>
+        <v>46051</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>46072</v>
+        <v>46061</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Sofia</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1324,17 +1326,17 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Stanmore Polymers</t>
+          <t>Trellisar</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Reading drift after ambient temperature rise</t>
+          <t>Firmware version query over API</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1343,16 +1345,16 @@
         </is>
       </c>
       <c r="F17" s="3" t="n">
-        <v>46070</v>
+        <v>46053</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>46075</v>
+        <v>46059</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
@@ -1361,7 +1363,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Sofia</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1378,17 +1380,17 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Harrowgate Cement</t>
+          <t>Quennick</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>4-20 mA output offset</t>
+          <t>Duplicate serial number on label</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1397,16 +1399,16 @@
         </is>
       </c>
       <c r="F18" s="3" t="n">
-        <v>46072</v>
+        <v>46054</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>46074</v>
+        <v>46058</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
@@ -1432,17 +1434,17 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Tallis Water Authority</t>
+          <t>Callowmere Packaging</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>False high-level alarm</t>
+          <t>Firmware update fails at 80 percent</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1451,30 +1453,30 @@
         </is>
       </c>
       <c r="F19" s="3" t="n">
-        <v>46073</v>
+        <v>46055</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>46077</v>
+        <v>46058</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1486,17 +1488,17 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Fenwick Aggregates</t>
+          <t>Sorrelby Water</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Cable gland leaking in washdown</t>
+          <t>Firmware version query over API</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1505,16 +1507,16 @@
         </is>
       </c>
       <c r="F20" s="3" t="n">
-        <v>46078</v>
+        <v>46056</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>46081</v>
+        <v>46062</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
@@ -1540,35 +1542,35 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Barrow Tide Ports</t>
+          <t>Tessivex</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>False high-level alarm</t>
+          <t>Unit reboots under brownout</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F21" s="3" t="n">
-        <v>46080</v>
+        <v>46059</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>46084</v>
+        <v>46075</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
@@ -1582,7 +1584,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1594,35 +1596,35 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Ironbridge Foundry</t>
+          <t>Tessivex</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Cable gland leaking in washdown</t>
+          <t>DIN clip broken on arrival</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F22" s="3" t="n">
-        <v>46080</v>
+        <v>46062</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>46083</v>
+        <v>46077</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
@@ -1631,12 +1633,12 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1648,17 +1650,17 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Barrow Tide Ports</t>
+          <t>Sorrelby Water</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Reading drift after ambient temperature rise</t>
+          <t>Question on mounting orientation</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1667,16 +1669,16 @@
         </is>
       </c>
       <c r="F23" s="3" t="n">
-        <v>46084</v>
+        <v>46063</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>46090</v>
+        <v>46075</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
@@ -1685,7 +1687,7 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Sofia</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -1702,17 +1704,17 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Fenwick Aggregates</t>
+          <t>Sorrelby Water</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Output chatter near target edge</t>
+          <t>Question on mounting orientation</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1721,16 +1723,16 @@
         </is>
       </c>
       <c r="F24" s="3" t="n">
-        <v>46084</v>
+        <v>46064</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>46088</v>
+        <v>46070</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
@@ -1756,49 +1758,49 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Meridian Industrial</t>
+          <t>Trellisar</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Firmware update failed mid-flash</t>
+          <t>Slow response on serial polling</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F25" s="3" t="n">
-        <v>46091</v>
+        <v>46066</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>46099</v>
+        <v>46079</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="I25" s="2" t="n">
         <v>10</v>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Sofia</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1810,17 +1812,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Quenby Plastics</t>
+          <t>Sorrelby Water</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Modbus register map question</t>
+          <t>Request for replacement terminal plugs</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1829,30 +1831,30 @@
         </is>
       </c>
       <c r="F26" s="3" t="n">
-        <v>46092</v>
+        <v>46069</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>46101</v>
+        <v>46085</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Marcus</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1864,35 +1866,35 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Stanmore Polymers</t>
+          <t>Tessivex</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Reading drift after ambient temperature rise</t>
+          <t>Unit reboots under brownout</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F27" s="3" t="n">
-        <v>46093</v>
+        <v>46071</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>46097</v>
+        <v>46080</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
@@ -1918,35 +1920,35 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Duvall Hydro</t>
+          <t>Sorrelby Water</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Firmware update failed mid-flash</t>
+          <t>Duplicate serial number on label</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F28" s="3" t="n">
-        <v>46094</v>
+        <v>46071</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>46095</v>
+        <v>46082</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
@@ -1972,17 +1974,17 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Brannock Refinery</t>
+          <t>Drossick</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Intermittent analog output dropout, unit BRN-0042</t>
+          <t>Wrong quick start card in box</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1991,16 +1993,16 @@
         </is>
       </c>
       <c r="F29" s="3" t="n">
-        <v>46099</v>
+        <v>46072</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>46100</v>
+        <v>46079</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
@@ -2026,17 +2028,17 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Delvecchio Packaging</t>
+          <t>Trellisar</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Unit fails self-test on power-up</t>
+          <t>Modbus register map out of date</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2045,20 +2047,20 @@
         </is>
       </c>
       <c r="F30" s="3" t="n">
-        <v>46101</v>
+        <v>46076</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>46106</v>
+        <v>46097</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -2080,35 +2082,35 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Hendricks Chemical</t>
+          <t>Sorrelby Water</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Echo loss on foam surface</t>
+          <t>Request for operating environment spec</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F31" s="3" t="n">
-        <v>46105</v>
+        <v>46076</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>46109</v>
+        <v>46080</v>
       </c>
       <c r="H31" s="2" t="n">
         <v>4</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
@@ -2117,12 +2119,12 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2134,49 +2136,49 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Ironbridge Foundry</t>
+          <t>Trellisar</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Output chatter near target edge</t>
+          <t>Status LED stays amber after boot</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F32" s="3" t="n">
-        <v>46108</v>
+        <v>46080</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>46115</v>
+        <v>46088</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Marcus</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2188,35 +2190,35 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Delvecchio Packaging</t>
+          <t>Kilnwarden Utilities</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Output chatter near target edge</t>
+          <t>Wrong quick start card in box</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F33" s="3" t="n">
-        <v>46111</v>
+        <v>46081</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>46114</v>
+        <v>46093</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
@@ -2225,12 +2227,12 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2242,35 +2244,35 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Quenby Plastics</t>
+          <t>Trellisar</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Configuration tool connection error</t>
+          <t>Unit fails self-test after power interruption</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F34" s="3" t="n">
-        <v>46111</v>
+        <v>46082</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>46114</v>
+        <v>46091</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
@@ -2296,49 +2298,49 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Brannock Refinery</t>
+          <t>Drossick</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Analog output dropout, second unit BRN-0067</t>
+          <t>Firmware update fails at 80 percent</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F35" s="3" t="n">
-        <v>46112</v>
+        <v>46084</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>46121</v>
+        <v>46099</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Marcus</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2350,39 +2352,39 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Delvecchio Packaging</t>
+          <t>Kilnwarden Utilities</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Output chatter near target edge</t>
+          <t>Clock drift between units</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F36" s="3" t="n">
-        <v>46115</v>
+        <v>46087</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>46120</v>
+        <v>46099</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -2404,39 +2406,39 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Marrowfield Foods</t>
+          <t>Kilnwarden Utilities</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>FieldSense 200</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Enclosure condensation</t>
+          <t>DIN clip broken on arrival</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="F37" s="3" t="n">
-        <v>46115</v>
+        <v>46089</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>46130</v>
+        <v>46090</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -2446,7 +2448,7 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2458,32 +2460,32 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Thornbury Power</t>
+          <t>Tharnwick Rail</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Modbus register map question</t>
+          <t>Ethernet link drops on managed switch</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F38" s="3" t="n">
-        <v>46115</v>
+        <v>46089</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>46120</v>
+        <v>46090</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I38" s="2" t="n">
         <v>5</v>
@@ -2500,7 +2502,7 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2512,35 +2514,35 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Brannock Refinery</t>
+          <t>Ivelmoor Group</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Erratic readings on three units, two process lines offline</t>
+          <t>Ethernet link drops on managed switch</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F39" s="3" t="n">
-        <v>46120</v>
+        <v>46090</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>46121</v>
+        <v>46096</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
@@ -2549,7 +2551,7 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Marcus</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -2566,17 +2568,17 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Coldharbour Logistics</t>
+          <t>Ivelmoor Group</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>FieldSense 200</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>PLC integration register mapping question</t>
+          <t>Request for replacement terminal plugs</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2585,20 +2587,20 @@
         </is>
       </c>
       <c r="F40" s="3" t="n">
-        <v>46126</v>
+        <v>46092</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>46142</v>
+        <v>46103</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -2620,17 +2622,17 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Tallis Water Authority</t>
+          <t>Tessivex</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Intermittent signal dropout</t>
+          <t>RS-485 termination setting unclear</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2639,16 +2641,16 @@
         </is>
       </c>
       <c r="F41" s="3" t="n">
-        <v>46126</v>
+        <v>46095</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>46130</v>
+        <v>46101</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
@@ -2674,17 +2676,17 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Hendricks Chemical</t>
+          <t>Tharnwick Rail</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Intermittent signal dropout</t>
+          <t>Firmware version query over API</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2693,25 +2695,25 @@
         </is>
       </c>
       <c r="F42" s="3" t="n">
-        <v>46129</v>
+        <v>46096</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>46141</v>
+        <v>46097</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Marcus</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
@@ -2728,39 +2730,39 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Meridian Industrial</t>
+          <t>Trellisar</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Modbus register map question</t>
+          <t>Unit fails self-test after power interruption</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="F43" s="3" t="n">
-        <v>46129</v>
+        <v>46099</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>46136</v>
+        <v>46100</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
@@ -2770,7 +2772,7 @@
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2782,39 +2784,39 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Coldharbour Logistics</t>
+          <t>Sorrelby Water</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>FieldSense 200</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Enclosure condensation</t>
+          <t>Ethernet link drops on managed switch</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F44" s="3" t="n">
-        <v>46133</v>
+        <v>46099</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>46139</v>
+        <v>46105</v>
       </c>
       <c r="H44" s="2" t="n">
         <v>6</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -2836,39 +2838,39 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Marrowfield Foods</t>
+          <t>Quennick</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>FieldSense 200</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Vibration baseline alarm too sensitive</t>
+          <t>Question on mounting orientation</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F45" s="3" t="n">
-        <v>46136</v>
+        <v>46101</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>46143</v>
+        <v>46105</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -2890,39 +2892,39 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Riverton Brewing</t>
+          <t>Tharnwick Rail</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>FieldSense 200</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Vibration baseline alarm too sensitive</t>
+          <t>Configuration lost after firmware update</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F46" s="3" t="n">
-        <v>46136</v>
+        <v>46105</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>46153</v>
+        <v>46105</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="I46" s="2" t="n">
         <v>10</v>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -2936,1137 +2938,1381 @@
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="51" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="54" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticket ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Opened Date</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Days Open</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>SLA Resolution Target (Days)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Within SLA</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Engineering Escalation</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Next Action</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>TKT-4146</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>Coldharbour Logistics</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>FieldSense 200</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>Commissioning wizard stalls</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Ivelmoor Group</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Intermittent RS-485 timeouts after panel rewiring</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>46072</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Termination and cable length checked; next step open</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4147</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Kilnwarden Utilities</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Static IP configuration steps</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F47" s="3" t="n">
-        <v>46139</v>
-      </c>
-      <c r="G47" s="3" t="n">
-        <v>46147</v>
-      </c>
-      <c r="H47" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="I47" s="2" t="n">
+      <c r="F3" s="3" t="n">
+        <v>46084</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4148</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Ivelmoor Group</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Register read interval shorter than 500 ms</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>46085</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="H4" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L47" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4147</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Riverton Brewing</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>FieldSense 200</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Commissioning wizard stalls</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Need a definitive firmware answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4149</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Sorrelby Water</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Modbus register map for holding registers</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F48" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="G48" s="3" t="n">
-        <v>46151</v>
-      </c>
-      <c r="H48" s="2" t="n">
+      <c r="F5" s="3" t="n">
+        <v>46085</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4150</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Pemberlith Foods</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>MX-3</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Operating humidity range</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>46086</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4151</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Callowmere Packaging</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>MX-3</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Replacement terminal plugs</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>46087</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4152</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Tharnwick Rail</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Static IP lost after power cycle</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>46088</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4153</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Drossick</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Quick start card references old web page</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>46089</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4154</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Quennick</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>MX-3</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Rated for 48 C ambient in summer?</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>46090</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Devon</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Confirm rating and any operating limits</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4155</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Tessivex</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>MX-3</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Recommended bus cable type</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>46090</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4156</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Kilnwarden Utilities</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>MX-3</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Mounting clearance around unit</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>46091</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4157</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Quennick</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>MX-3</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Operating limits at sustained high ambient</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>46092</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Devon</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Confirm rating and any operating limits</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4158</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Sorrelby Water</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Modbus register scaling for status word</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>46092</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4159</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Trellisar</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Modbus TCP support in addition to RTU</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>46093</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Sofia</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Confirm roadmap position</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4160</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Oskerry Systems</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Operating temperature for outdoor cabinet</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>46093</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4161</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Pemberlith Foods</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Default web password reset</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>46094</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4162</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Callowmere Packaging</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Firmware version check procedure</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>46095</v>
+      </c>
+      <c r="G18" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="I48" s="2" t="n">
+      <c r="H18" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4163</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Tharnwick Rail</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>MX-3</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Label placement for asset tags</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>46096</v>
+      </c>
+      <c r="G19" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr">
+      <c r="H19" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4164</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Quennick</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>MX-3</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Support horizon for firmware 2.4.1</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>46097</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>Sofia</t>
         </is>
       </c>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4148</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>Ironbridge Foundry</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>ProximaSense X4</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>Output chatter near target edge</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Needs a firmware lifecycle policy answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4165</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Drossick</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>DHCP lease renewal behaviour</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F49" s="3" t="n">
-        <v>46141</v>
-      </c>
-      <c r="G49" s="3" t="n">
-        <v>46156</v>
-      </c>
-      <c r="H49" s="2" t="n">
+      <c r="F21" s="3" t="n">
+        <v>46097</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="H21" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="I49" s="2" t="n">
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4166</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Trellisar</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Status LED dimmer than on other units</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>46099</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Devon</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Assess whether a replacement is warranted</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4167</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Hessanby Dynamics</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Commissioning: unit not found on network</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>46101</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H23" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J49" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K49" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L49" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4149</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Quenby Plastics</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev B</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>Intermittent signal dropout</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="n">
-        <v>46143</v>
-      </c>
-      <c r="G50" s="3" t="n">
-        <v>46150</v>
-      </c>
-      <c r="H50" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="I50" s="2" t="n">
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Walk through discovery setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4168</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Hessanby Dynamics</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Commissioning: RS-485 address assignment</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>46104</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J50" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K50" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L50" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4150</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>Stanmore Polymers</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev B</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>4-20 mA output offset</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="n">
-        <v>46148</v>
-      </c>
-      <c r="G51" s="3" t="n">
-        <v>46162</v>
-      </c>
-      <c r="H51" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="I51" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J51" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K51" s="2" t="inlineStr">
-        <is>
-          <t>Sofia</t>
-        </is>
-      </c>
-      <c r="L51" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4151</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>Duvall Hydro</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev B</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>Firmware update failed mid-flash</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="n">
-        <v>46150</v>
-      </c>
-      <c r="G52" s="3" t="n">
-        <v>46160</v>
-      </c>
-      <c r="H52" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="I52" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K52" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L52" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4152</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>Whitlow Dairy</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev B</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>Firmware update failed mid-flash</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F53" s="3" t="n">
-        <v>46155</v>
-      </c>
-      <c r="G53" s="3" t="n">
-        <v>46165</v>
-      </c>
-      <c r="H53" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="I53" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J53" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K53" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L53" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4153</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>Barrow Tide Ports</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev B</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>False high-level alarm</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="n">
-        <v>46156</v>
-      </c>
-      <c r="G54" s="3" t="n">
-        <v>46164</v>
-      </c>
-      <c r="H54" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="I54" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J54" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K54" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L54" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4154</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>Upton Cold Storage</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>FieldSense 200</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>Dashboard shows stale readings</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F55" s="3" t="n">
-        <v>46156</v>
-      </c>
-      <c r="G55" s="3" t="n">
-        <v>46161</v>
-      </c>
-      <c r="H55" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I55" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J55" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K55" s="2" t="inlineStr">
-        <is>
-          <t>Sofia</t>
-        </is>
-      </c>
-      <c r="L55" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4155</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>Upton Cold Storage</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>FieldSense 200</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>Vibration baseline alarm too sensitive</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="n">
-        <v>46157</v>
-      </c>
-      <c r="G56" s="3" t="n">
-        <v>46161</v>
-      </c>
-      <c r="H56" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="I56" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J56" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K56" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L56" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4156</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>Carver Automation</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>FieldSense 200</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>Demo unit not reporting after firmware configuration</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F57" s="3" t="n">
-        <v>46160</v>
-      </c>
-      <c r="G57" s="3" t="n">
-        <v>46169</v>
-      </c>
-      <c r="H57" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="I57" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J57" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K57" s="2" t="inlineStr">
-        <is>
-          <t>Sofia</t>
-        </is>
-      </c>
-      <c r="L57" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4157</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>Fenwick Aggregates</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>ProximaSense X4</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>Cable gland leaking in washdown</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F58" s="3" t="n">
-        <v>46161</v>
-      </c>
-      <c r="G58" s="3" t="n">
-        <v>46167</v>
-      </c>
-      <c r="H58" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="I58" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J58" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K58" s="2" t="inlineStr">
-        <is>
-          <t>Marcus</t>
-        </is>
-      </c>
-      <c r="L58" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4158</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>Harrowgate Cement</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev C</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>Modbus register map question</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F59" s="3" t="n">
-        <v>46161</v>
-      </c>
-      <c r="G59" s="3" t="n">
-        <v>46168</v>
-      </c>
-      <c r="H59" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="I59" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J59" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K59" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L59" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4159</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>Hendricks Chemical</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev C</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>Level reading lags during rapid tank fill</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F60" s="3" t="n">
-        <v>46162</v>
-      </c>
-      <c r="G60" s="3" t="n">
-        <v>46170</v>
-      </c>
-      <c r="H60" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="I60" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J60" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K60" s="2" t="inlineStr">
-        <is>
-          <t>Sofia</t>
-        </is>
-      </c>
-      <c r="L60" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4160</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>Ironbridge Foundry</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>ProximaSense X4</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>Replacement mounting bracket request</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F61" s="3" t="n">
-        <v>46163</v>
-      </c>
-      <c r="G61" s="3" t="n">
-        <v>46171</v>
-      </c>
-      <c r="H61" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="I61" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J61" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K61" s="2" t="inlineStr">
-        <is>
-          <t>Sofia</t>
-        </is>
-      </c>
-      <c r="L61" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4161</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>Marrowfield Foods</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>FieldSense 200</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>Vibration baseline alarm too sensitive</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F62" s="3" t="n">
-        <v>46163</v>
-      </c>
-      <c r="G62" s="3" t="n">
-        <v>46171</v>
-      </c>
-      <c r="H62" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="I62" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J62" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K62" s="2" t="inlineStr">
-        <is>
-          <t>Marcus</t>
-        </is>
-      </c>
-      <c r="L62" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4162</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>Duvall Hydro</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev B</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>Firmware update failed mid-flash</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F63" s="3" t="n">
-        <v>46164</v>
-      </c>
-      <c r="G63" s="3" t="n">
-        <v>46171</v>
-      </c>
-      <c r="H63" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="I63" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J63" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K63" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L63" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4163</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>Ironbridge Foundry</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>ProximaSense X4</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>Output chatter near target edge</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F64" s="3" t="n">
-        <v>46164</v>
-      </c>
-      <c r="G64" s="3" t="n">
-        <v>46171</v>
-      </c>
-      <c r="H64" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="I64" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J64" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K64" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L64" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4164</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>Marrowfield Foods</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>FieldSense 200</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>Dashboard shows stale readings</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F65" s="3" t="n">
-        <v>46164</v>
-      </c>
-      <c r="G65" s="3" t="n">
-        <v>46171</v>
-      </c>
-      <c r="H65" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="I65" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J65" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K65" s="2" t="inlineStr">
-        <is>
-          <t>Marcus</t>
-        </is>
-      </c>
-      <c r="L65" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4165</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>Tallis Water Authority</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev C</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>Echo loss on foam surface</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F66" s="3" t="n">
-        <v>46168</v>
-      </c>
-      <c r="G66" s="3" t="n">
-        <v>46171</v>
-      </c>
-      <c r="H66" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I66" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J66" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K66" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L66" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4166</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>Ironbridge Foundry</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>ProximaSense X4</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>Unit fails self-test on power-up</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="n">
-        <v>46170</v>
-      </c>
-      <c r="G67" s="3" t="n">
-        <v>46171</v>
-      </c>
-      <c r="H67" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I67" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J67" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K67" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L67" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Send addressing guide</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: rename the company and regenerate the corpus (#123)
Widget Makers Incorporated shares its name with a real manufacturer, and
several names invented inside the corpus did too. The generation prompts,
roster, and office guidance now name Main St Widget Foundry LLC, keep its
products deliberately vague, and forbid real company and product names.

The transcripts, office files, and store are regenerated, with every
invented name checked against a web search and replaced where it was
real. The tests, README examples, frontend fixtures, and the record of
planted imperfections follow the new corpus.

Closes #122
</commit_message>
<xml_diff>
--- a/data/office/support-ticket-sla-log.xlsx
+++ b/data/office/support-ticket-sla-log.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resolved Tickets" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resolved Tickets" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Tickets" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -427,19 +429,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="47" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
   </cols>
@@ -514,32 +516,32 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Fenwick Aggregates</t>
+          <t>Ivelmoor Group</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Unit fails self-test on power-up</t>
+          <t>RS-485 termination setting unclear</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>46023</v>
+        <v>46024</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>46027</v>
+        <v>46026</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>5</v>
@@ -551,12 +553,12 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -568,32 +570,32 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Harrowgate Cement</t>
+          <t>Quennick</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Intermittent signal dropout</t>
+          <t>Clock drift between units</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>46027</v>
+        <v>46025</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>46037</v>
+        <v>46031</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>10</v>
@@ -605,12 +607,12 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Sofia</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -622,35 +624,35 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Fenwick Aggregates</t>
+          <t>Trellisar</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Output chatter near target edge</t>
+          <t>Request for operating environment spec</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
+        <v>46027</v>
+      </c>
+      <c r="G4" s="3" t="n">
         <v>46029</v>
       </c>
-      <c r="G4" s="3" t="n">
-        <v>46033</v>
-      </c>
       <c r="H4" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -664,7 +666,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -676,35 +678,35 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Fenwick Aggregates</t>
+          <t>Tharnwick Rail</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Replacement mounting bracket request</t>
+          <t>Firmware update fails at 80 percent</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>46031</v>
+        <v>46029</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>46034</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
@@ -713,12 +715,12 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -730,17 +732,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Kessler Paper Mill</t>
+          <t>Tessivex</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Reading drift after ambient temperature rise</t>
+          <t>Slow response on serial polling</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -749,16 +751,16 @@
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>46031</v>
+        <v>46032</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>46035</v>
+        <v>46038</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -767,12 +769,12 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -784,35 +786,35 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Thornbury Power</t>
+          <t>Pemberlith Foods</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Echo loss on foam surface</t>
+          <t>Unit fails self-test after power interruption</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>46031</v>
+        <v>46035</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>46033</v>
+        <v>46044</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
@@ -838,35 +840,35 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Barrow Tide Ports</t>
+          <t>Quennick</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Configuration tool connection error</t>
+          <t>Request for replacement terminal plugs</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
         <v>46034</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>46035</v>
+        <v>46037</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -875,12 +877,12 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -892,49 +894,49 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Grayson Textiles</t>
+          <t>Pemberlith Foods</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Reading drift after ambient temperature rise</t>
+          <t>Question on mounting orientation</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>46043</v>
+        <v>46036</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>46047</v>
+        <v>46048</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Marcus</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -946,35 +948,35 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Sable Creek Gas</t>
+          <t>Pemberlith Foods</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Calibration offset after install</t>
+          <t>Unit fails self-test after power interruption</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46045</v>
+        <v>46038</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>46049</v>
+        <v>46039</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
@@ -988,7 +990,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1000,35 +1002,35 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Thornbury Power</t>
+          <t>Pemberlith Foods</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Intermittent signal dropout</t>
+          <t>Configuration lost after firmware update</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="F11" s="3" t="n">
-        <v>46049</v>
+        <v>46041</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>46053</v>
+        <v>46043</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
@@ -1037,12 +1039,12 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1054,29 +1056,29 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Grayson Textiles</t>
+          <t>Sorrelby Water</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Firmware update failed mid-flash</t>
+          <t>Unit reboots under brownout</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F12" s="3" t="n">
-        <v>46055</v>
+        <v>46042</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>46059</v>
+        <v>46046</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>4</v>
@@ -1091,12 +1093,12 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1108,49 +1110,49 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Stanmore Polymers</t>
+          <t>Tharnwick Rail</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Echo loss on foam surface</t>
+          <t>Bus address conflict on commissioning</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F13" s="3" t="n">
-        <v>46059</v>
+        <v>46044</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>46063</v>
+        <v>46053</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Sofia</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1162,35 +1164,35 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Delvecchio Packaging</t>
+          <t>Callowmere Packaging</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Output chatter near target edge</t>
+          <t>Unit reboots under brownout</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F14" s="3" t="n">
-        <v>46063</v>
+        <v>46047</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>46069</v>
+        <v>46049</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
@@ -1199,12 +1201,12 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1216,49 +1218,49 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Sable Creek Gas</t>
+          <t>Ivelmoor Group</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>4-20 mA output offset</t>
+          <t>Firmware update fails at 80 percent</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F15" s="3" t="n">
-        <v>46065</v>
+        <v>46049</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>46069</v>
+        <v>46058</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Sofia</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1270,49 +1272,49 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Sable Creek Gas</t>
+          <t>Kilnwarden Utilities</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Firmware update failed mid-flash</t>
+          <t>Firmware version query over API</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
-        <v>46066</v>
+        <v>46051</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>46072</v>
+        <v>46061</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Sofia</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1324,17 +1326,17 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Stanmore Polymers</t>
+          <t>Trellisar</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Reading drift after ambient temperature rise</t>
+          <t>Firmware version query over API</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1343,16 +1345,16 @@
         </is>
       </c>
       <c r="F17" s="3" t="n">
-        <v>46070</v>
+        <v>46053</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>46075</v>
+        <v>46059</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
@@ -1361,7 +1363,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Sofia</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1378,17 +1380,17 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Harrowgate Cement</t>
+          <t>Quennick</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>4-20 mA output offset</t>
+          <t>Duplicate serial number on label</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1397,16 +1399,16 @@
         </is>
       </c>
       <c r="F18" s="3" t="n">
-        <v>46072</v>
+        <v>46054</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>46074</v>
+        <v>46058</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
@@ -1432,17 +1434,17 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Tallis Water Authority</t>
+          <t>Callowmere Packaging</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>False high-level alarm</t>
+          <t>Firmware update fails at 80 percent</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1451,30 +1453,30 @@
         </is>
       </c>
       <c r="F19" s="3" t="n">
-        <v>46073</v>
+        <v>46055</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>46077</v>
+        <v>46058</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1486,17 +1488,17 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Fenwick Aggregates</t>
+          <t>Sorrelby Water</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Cable gland leaking in washdown</t>
+          <t>Firmware version query over API</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1505,16 +1507,16 @@
         </is>
       </c>
       <c r="F20" s="3" t="n">
-        <v>46078</v>
+        <v>46056</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>46081</v>
+        <v>46062</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
@@ -1540,35 +1542,35 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Barrow Tide Ports</t>
+          <t>Tessivex</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>False high-level alarm</t>
+          <t>Unit reboots under brownout</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F21" s="3" t="n">
-        <v>46080</v>
+        <v>46059</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>46084</v>
+        <v>46075</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
@@ -1582,7 +1584,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1594,35 +1596,35 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Ironbridge Foundry</t>
+          <t>Tessivex</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Cable gland leaking in washdown</t>
+          <t>DIN clip broken on arrival</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F22" s="3" t="n">
-        <v>46080</v>
+        <v>46062</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>46083</v>
+        <v>46077</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
@@ -1631,12 +1633,12 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1648,17 +1650,17 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Barrow Tide Ports</t>
+          <t>Sorrelby Water</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Reading drift after ambient temperature rise</t>
+          <t>Question on mounting orientation</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1667,16 +1669,16 @@
         </is>
       </c>
       <c r="F23" s="3" t="n">
-        <v>46084</v>
+        <v>46063</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>46090</v>
+        <v>46075</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
@@ -1685,7 +1687,7 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Sofia</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -1702,17 +1704,17 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Fenwick Aggregates</t>
+          <t>Sorrelby Water</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Output chatter near target edge</t>
+          <t>Question on mounting orientation</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1721,16 +1723,16 @@
         </is>
       </c>
       <c r="F24" s="3" t="n">
-        <v>46084</v>
+        <v>46064</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>46088</v>
+        <v>46070</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
@@ -1756,49 +1758,49 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Meridian Industrial</t>
+          <t>Trellisar</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Firmware update failed mid-flash</t>
+          <t>Slow response on serial polling</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F25" s="3" t="n">
-        <v>46091</v>
+        <v>46066</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>46099</v>
+        <v>46079</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="I25" s="2" t="n">
         <v>10</v>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Sofia</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1810,17 +1812,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Quenby Plastics</t>
+          <t>Sorrelby Water</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Modbus register map question</t>
+          <t>Request for replacement terminal plugs</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1829,30 +1831,30 @@
         </is>
       </c>
       <c r="F26" s="3" t="n">
-        <v>46092</v>
+        <v>46069</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>46101</v>
+        <v>46085</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Marcus</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1864,35 +1866,35 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Stanmore Polymers</t>
+          <t>Tessivex</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Reading drift after ambient temperature rise</t>
+          <t>Unit reboots under brownout</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F27" s="3" t="n">
-        <v>46093</v>
+        <v>46071</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>46097</v>
+        <v>46080</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
@@ -1918,35 +1920,35 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Duvall Hydro</t>
+          <t>Sorrelby Water</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Firmware update failed mid-flash</t>
+          <t>Duplicate serial number on label</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F28" s="3" t="n">
-        <v>46094</v>
+        <v>46071</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>46095</v>
+        <v>46082</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
@@ -1972,17 +1974,17 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Brannock Refinery</t>
+          <t>Drossick</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Intermittent analog output dropout, unit BRN-0042</t>
+          <t>Wrong quick start card in box</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1991,16 +1993,16 @@
         </is>
       </c>
       <c r="F29" s="3" t="n">
-        <v>46099</v>
+        <v>46072</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>46100</v>
+        <v>46079</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
@@ -2026,17 +2028,17 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Delvecchio Packaging</t>
+          <t>Trellisar</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Unit fails self-test on power-up</t>
+          <t>Modbus register map out of date</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2045,20 +2047,20 @@
         </is>
       </c>
       <c r="F30" s="3" t="n">
-        <v>46101</v>
+        <v>46076</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>46106</v>
+        <v>46097</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -2080,35 +2082,35 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Hendricks Chemical</t>
+          <t>Sorrelby Water</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Echo loss on foam surface</t>
+          <t>Request for operating environment spec</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F31" s="3" t="n">
-        <v>46105</v>
+        <v>46076</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>46109</v>
+        <v>46080</v>
       </c>
       <c r="H31" s="2" t="n">
         <v>4</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
@@ -2117,12 +2119,12 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2134,49 +2136,49 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Ironbridge Foundry</t>
+          <t>Trellisar</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Output chatter near target edge</t>
+          <t>Status LED stays amber after boot</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F32" s="3" t="n">
-        <v>46108</v>
+        <v>46080</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>46115</v>
+        <v>46088</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Marcus</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2188,35 +2190,35 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Delvecchio Packaging</t>
+          <t>Kilnwarden Utilities</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Output chatter near target edge</t>
+          <t>Wrong quick start card in box</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F33" s="3" t="n">
-        <v>46111</v>
+        <v>46081</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>46114</v>
+        <v>46093</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
@@ -2225,12 +2227,12 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2242,35 +2244,35 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Quenby Plastics</t>
+          <t>Trellisar</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Configuration tool connection error</t>
+          <t>Unit fails self-test after power interruption</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F34" s="3" t="n">
-        <v>46111</v>
+        <v>46082</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>46114</v>
+        <v>46091</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
@@ -2296,49 +2298,49 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Brannock Refinery</t>
+          <t>Drossick</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Analog output dropout, second unit BRN-0067</t>
+          <t>Firmware update fails at 80 percent</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F35" s="3" t="n">
-        <v>46112</v>
+        <v>46084</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>46121</v>
+        <v>46099</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Marcus</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2350,39 +2352,39 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Delvecchio Packaging</t>
+          <t>Kilnwarden Utilities</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>ProximaSense X4</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Output chatter near target edge</t>
+          <t>Clock drift between units</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F36" s="3" t="n">
-        <v>46115</v>
+        <v>46087</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>46120</v>
+        <v>46099</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -2404,39 +2406,39 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Marrowfield Foods</t>
+          <t>Kilnwarden Utilities</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>FieldSense 200</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Enclosure condensation</t>
+          <t>DIN clip broken on arrival</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="F37" s="3" t="n">
-        <v>46115</v>
+        <v>46089</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>46130</v>
+        <v>46090</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -2446,7 +2448,7 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2458,32 +2460,32 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Thornbury Power</t>
+          <t>Tharnwick Rail</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Modbus register map question</t>
+          <t>Ethernet link drops on managed switch</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F38" s="3" t="n">
-        <v>46115</v>
+        <v>46089</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>46120</v>
+        <v>46090</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I38" s="2" t="n">
         <v>5</v>
@@ -2500,7 +2502,7 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2512,35 +2514,35 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Brannock Refinery</t>
+          <t>Ivelmoor Group</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Erratic readings on three units, two process lines offline</t>
+          <t>Ethernet link drops on managed switch</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F39" s="3" t="n">
-        <v>46120</v>
+        <v>46090</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>46121</v>
+        <v>46096</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
@@ -2549,7 +2551,7 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Marcus</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -2566,17 +2568,17 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Coldharbour Logistics</t>
+          <t>Ivelmoor Group</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>FieldSense 200</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>PLC integration register mapping question</t>
+          <t>Request for replacement terminal plugs</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2585,20 +2587,20 @@
         </is>
       </c>
       <c r="F40" s="3" t="n">
-        <v>46126</v>
+        <v>46092</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>46142</v>
+        <v>46103</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -2620,17 +2622,17 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Tallis Water Authority</t>
+          <t>Tessivex</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Intermittent signal dropout</t>
+          <t>RS-485 termination setting unclear</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2639,16 +2641,16 @@
         </is>
       </c>
       <c r="F41" s="3" t="n">
-        <v>46126</v>
+        <v>46095</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>46130</v>
+        <v>46101</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
@@ -2674,17 +2676,17 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Hendricks Chemical</t>
+          <t>Tharnwick Rail</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev B</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Intermittent signal dropout</t>
+          <t>Firmware version query over API</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2693,25 +2695,25 @@
         </is>
       </c>
       <c r="F42" s="3" t="n">
-        <v>46129</v>
+        <v>46096</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>46141</v>
+        <v>46097</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Marcus</t>
+          <t>Theo</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
@@ -2728,39 +2730,39 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Meridian Industrial</t>
+          <t>Trellisar</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>XT-9 Rev C</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Modbus register map question</t>
+          <t>Unit fails self-test after power interruption</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="F43" s="3" t="n">
-        <v>46129</v>
+        <v>46099</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>46136</v>
+        <v>46100</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
@@ -2770,7 +2772,7 @@
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2782,39 +2784,39 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Coldharbour Logistics</t>
+          <t>Sorrelby Water</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>FieldSense 200</t>
+          <t>GX-7</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Enclosure condensation</t>
+          <t>Ethernet link drops on managed switch</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F44" s="3" t="n">
-        <v>46133</v>
+        <v>46099</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>46139</v>
+        <v>46105</v>
       </c>
       <c r="H44" s="2" t="n">
         <v>6</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -2836,39 +2838,39 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Marrowfield Foods</t>
+          <t>Quennick</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>FieldSense 200</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Vibration baseline alarm too sensitive</t>
+          <t>Question on mounting orientation</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F45" s="3" t="n">
-        <v>46136</v>
+        <v>46101</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>46143</v>
+        <v>46105</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -2890,39 +2892,39 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Riverton Brewing</t>
+          <t>Tharnwick Rail</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>FieldSense 200</t>
+          <t>MX-3</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Vibration baseline alarm too sensitive</t>
+          <t>Configuration lost after firmware update</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F46" s="3" t="n">
-        <v>46136</v>
+        <v>46105</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>46153</v>
+        <v>46105</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="I46" s="2" t="n">
         <v>10</v>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -2936,1137 +2938,1381 @@
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="51" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="54" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticket ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Opened Date</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Days Open</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>SLA Resolution Target (Days)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Within SLA</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Engineering Escalation</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Next Action</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>TKT-4146</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>Coldharbour Logistics</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>FieldSense 200</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>Commissioning wizard stalls</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Ivelmoor Group</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Intermittent RS-485 timeouts after panel rewiring</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>46072</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Termination and cable length checked; next step open</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4147</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Kilnwarden Utilities</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Static IP configuration steps</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F47" s="3" t="n">
-        <v>46139</v>
-      </c>
-      <c r="G47" s="3" t="n">
-        <v>46147</v>
-      </c>
-      <c r="H47" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="I47" s="2" t="n">
+      <c r="F3" s="3" t="n">
+        <v>46084</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4148</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Ivelmoor Group</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Register read interval shorter than 500 ms</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>46085</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="H4" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L47" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4147</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Riverton Brewing</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>FieldSense 200</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Commissioning wizard stalls</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Need a definitive firmware answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4149</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Sorrelby Water</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Modbus register map for holding registers</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F48" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="G48" s="3" t="n">
-        <v>46151</v>
-      </c>
-      <c r="H48" s="2" t="n">
+      <c r="F5" s="3" t="n">
+        <v>46085</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4150</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Pemberlith Foods</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>MX-3</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Operating humidity range</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>46086</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4151</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Callowmere Packaging</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>MX-3</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Replacement terminal plugs</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>46087</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4152</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Tharnwick Rail</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Static IP lost after power cycle</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>46088</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4153</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Drossick</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Quick start card references old web page</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>46089</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4154</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Quennick</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>MX-3</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Rated for 48 C ambient in summer?</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>46090</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Devon</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Confirm rating and any operating limits</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4155</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Tessivex</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>MX-3</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Recommended bus cable type</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>46090</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4156</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Kilnwarden Utilities</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>MX-3</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Mounting clearance around unit</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>46091</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4157</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Quennick</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>MX-3</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Operating limits at sustained high ambient</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>46092</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Devon</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Confirm rating and any operating limits</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4158</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Sorrelby Water</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Modbus register scaling for status word</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>46092</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4159</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Trellisar</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Modbus TCP support in addition to RTU</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>46093</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Sofia</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Confirm roadmap position</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4160</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Oskerry Systems</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Operating temperature for outdoor cabinet</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>46093</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4161</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Pemberlith Foods</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Default web password reset</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>46094</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4162</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Callowmere Packaging</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Firmware version check procedure</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>46095</v>
+      </c>
+      <c r="G18" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="I48" s="2" t="n">
+      <c r="H18" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4163</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Tharnwick Rail</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>MX-3</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Label placement for asset tags</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>46096</v>
+      </c>
+      <c r="G19" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr">
+      <c r="H19" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4164</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Quennick</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>MX-3</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Support horizon for firmware 2.4.1</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>46097</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>Sofia</t>
         </is>
       </c>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4148</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>Ironbridge Foundry</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>ProximaSense X4</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>Output chatter near target edge</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Needs a firmware lifecycle policy answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4165</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Drossick</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>DHCP lease renewal behaviour</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F49" s="3" t="n">
-        <v>46141</v>
-      </c>
-      <c r="G49" s="3" t="n">
-        <v>46156</v>
-      </c>
-      <c r="H49" s="2" t="n">
+      <c r="F21" s="3" t="n">
+        <v>46097</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="H21" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="I49" s="2" t="n">
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Answer from documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4166</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Trellisar</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Status LED dimmer than on other units</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>46099</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Devon</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Assess whether a replacement is warranted</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4167</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Hessanby Dynamics</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Commissioning: unit not found on network</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>46101</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H23" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J49" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K49" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L49" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4149</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Quenby Plastics</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev B</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>Intermittent signal dropout</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="n">
-        <v>46143</v>
-      </c>
-      <c r="G50" s="3" t="n">
-        <v>46150</v>
-      </c>
-      <c r="H50" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="I50" s="2" t="n">
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Walk through discovery setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TKT-4168</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Hessanby Dynamics</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>GX-7</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Commissioning: RS-485 address assignment</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>46104</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J50" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K50" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L50" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4150</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>Stanmore Polymers</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev B</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>4-20 mA output offset</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="n">
-        <v>46148</v>
-      </c>
-      <c r="G51" s="3" t="n">
-        <v>46162</v>
-      </c>
-      <c r="H51" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="I51" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J51" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K51" s="2" t="inlineStr">
-        <is>
-          <t>Sofia</t>
-        </is>
-      </c>
-      <c r="L51" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4151</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>Duvall Hydro</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev B</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>Firmware update failed mid-flash</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="n">
-        <v>46150</v>
-      </c>
-      <c r="G52" s="3" t="n">
-        <v>46160</v>
-      </c>
-      <c r="H52" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="I52" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K52" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L52" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4152</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>Whitlow Dairy</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev B</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>Firmware update failed mid-flash</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F53" s="3" t="n">
-        <v>46155</v>
-      </c>
-      <c r="G53" s="3" t="n">
-        <v>46165</v>
-      </c>
-      <c r="H53" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="I53" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J53" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K53" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L53" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4153</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>Barrow Tide Ports</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev B</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>False high-level alarm</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="n">
-        <v>46156</v>
-      </c>
-      <c r="G54" s="3" t="n">
-        <v>46164</v>
-      </c>
-      <c r="H54" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="I54" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J54" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K54" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L54" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4154</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>Upton Cold Storage</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>FieldSense 200</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>Dashboard shows stale readings</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F55" s="3" t="n">
-        <v>46156</v>
-      </c>
-      <c r="G55" s="3" t="n">
-        <v>46161</v>
-      </c>
-      <c r="H55" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I55" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J55" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K55" s="2" t="inlineStr">
-        <is>
-          <t>Sofia</t>
-        </is>
-      </c>
-      <c r="L55" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4155</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>Upton Cold Storage</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>FieldSense 200</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>Vibration baseline alarm too sensitive</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="n">
-        <v>46157</v>
-      </c>
-      <c r="G56" s="3" t="n">
-        <v>46161</v>
-      </c>
-      <c r="H56" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="I56" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J56" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K56" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L56" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4156</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>Carver Automation</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>FieldSense 200</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>Demo unit not reporting after firmware configuration</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F57" s="3" t="n">
-        <v>46160</v>
-      </c>
-      <c r="G57" s="3" t="n">
-        <v>46169</v>
-      </c>
-      <c r="H57" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="I57" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J57" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K57" s="2" t="inlineStr">
-        <is>
-          <t>Sofia</t>
-        </is>
-      </c>
-      <c r="L57" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4157</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>Fenwick Aggregates</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>ProximaSense X4</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>Cable gland leaking in washdown</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F58" s="3" t="n">
-        <v>46161</v>
-      </c>
-      <c r="G58" s="3" t="n">
-        <v>46167</v>
-      </c>
-      <c r="H58" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="I58" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J58" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K58" s="2" t="inlineStr">
-        <is>
-          <t>Marcus</t>
-        </is>
-      </c>
-      <c r="L58" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4158</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>Harrowgate Cement</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev C</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>Modbus register map question</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F59" s="3" t="n">
-        <v>46161</v>
-      </c>
-      <c r="G59" s="3" t="n">
-        <v>46168</v>
-      </c>
-      <c r="H59" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="I59" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J59" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K59" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L59" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4159</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>Hendricks Chemical</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev C</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>Level reading lags during rapid tank fill</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F60" s="3" t="n">
-        <v>46162</v>
-      </c>
-      <c r="G60" s="3" t="n">
-        <v>46170</v>
-      </c>
-      <c r="H60" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="I60" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J60" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K60" s="2" t="inlineStr">
-        <is>
-          <t>Sofia</t>
-        </is>
-      </c>
-      <c r="L60" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4160</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>Ironbridge Foundry</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>ProximaSense X4</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>Replacement mounting bracket request</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F61" s="3" t="n">
-        <v>46163</v>
-      </c>
-      <c r="G61" s="3" t="n">
-        <v>46171</v>
-      </c>
-      <c r="H61" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="I61" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J61" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K61" s="2" t="inlineStr">
-        <is>
-          <t>Sofia</t>
-        </is>
-      </c>
-      <c r="L61" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4161</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>Marrowfield Foods</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>FieldSense 200</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>Vibration baseline alarm too sensitive</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F62" s="3" t="n">
-        <v>46163</v>
-      </c>
-      <c r="G62" s="3" t="n">
-        <v>46171</v>
-      </c>
-      <c r="H62" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="I62" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J62" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K62" s="2" t="inlineStr">
-        <is>
-          <t>Marcus</t>
-        </is>
-      </c>
-      <c r="L62" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4162</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>Duvall Hydro</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev B</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>Firmware update failed mid-flash</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F63" s="3" t="n">
-        <v>46164</v>
-      </c>
-      <c r="G63" s="3" t="n">
-        <v>46171</v>
-      </c>
-      <c r="H63" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="I63" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J63" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K63" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L63" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4163</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>Ironbridge Foundry</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>ProximaSense X4</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>Output chatter near target edge</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F64" s="3" t="n">
-        <v>46164</v>
-      </c>
-      <c r="G64" s="3" t="n">
-        <v>46171</v>
-      </c>
-      <c r="H64" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="I64" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J64" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K64" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L64" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4164</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>Marrowfield Foods</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>FieldSense 200</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>Dashboard shows stale readings</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F65" s="3" t="n">
-        <v>46164</v>
-      </c>
-      <c r="G65" s="3" t="n">
-        <v>46171</v>
-      </c>
-      <c r="H65" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="I65" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J65" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K65" s="2" t="inlineStr">
-        <is>
-          <t>Marcus</t>
-        </is>
-      </c>
-      <c r="L65" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4165</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>Tallis Water Authority</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>XT-9 Rev C</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>Echo loss on foam surface</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F66" s="3" t="n">
-        <v>46168</v>
-      </c>
-      <c r="G66" s="3" t="n">
-        <v>46171</v>
-      </c>
-      <c r="H66" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I66" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J66" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K66" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L66" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>TKT-4166</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>Ironbridge Foundry</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>ProximaSense X4</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>Unit fails self-test on power-up</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="n">
-        <v>46170</v>
-      </c>
-      <c r="G67" s="3" t="n">
-        <v>46171</v>
-      </c>
-      <c r="H67" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I67" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J67" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K67" s="2" t="inlineStr">
-        <is>
-          <t>Theo</t>
-        </is>
-      </c>
-      <c r="L67" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Send addressing guide</t>
         </is>
       </c>
     </row>

</xml_diff>